<commit_message>
CHANAS Last update for the prestataire
</commit_message>
<xml_diff>
--- a/chanas/presta/media/prestataire_soins2.xlsx
+++ b/chanas/presta/media/prestataire_soins2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antboy/Desktop/PWC/CODE/venv/chanas_2/chanas/presta/media/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE199527-EED4-F54F-A139-56FE28AE7A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1C8763-7689-F241-B1EA-466E1CCDA123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{DAEB2858-4AB9-DC42-BCCA-AA77F40B5715}"/>
   </bookViews>
@@ -1598,9 +1598,6 @@
     <t>MAROUA</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <r>
       <t> </t>
     </r>
@@ -1647,6 +1644,9 @@
   </si>
   <si>
     <t>FOUNDATION</t>
+  </si>
+  <si>
+    <t>TYPE</t>
   </si>
 </sst>
 </file>
@@ -1797,7 +1797,7 @@
     <tableColumn id="2" xr3:uid="{2622A07C-27E5-7342-A004-FC36A3C08F04}" name="PRESTATAIRES" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{0513F6E7-602A-ED46-8CFE-B9790B9A6BD2}" name="LIEU" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{7CD384D9-9904-2640-B4D9-D31547083864}" name="TELEPHONE"/>
-    <tableColumn id="5" xr3:uid="{DFD4B9DD-90BB-F949-8950-AACF1FD0E6AD}" name="Type"/>
+    <tableColumn id="5" xr3:uid="{DFD4B9DD-90BB-F949-8950-AACF1FD0E6AD}" name="TYPE"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2144,7 +2144,7 @@
         <v>5</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -4769,7 +4769,7 @@
         <v>39</v>
       </c>
       <c r="E167" s="1" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.2">
@@ -4786,7 +4786,7 @@
         <v>41</v>
       </c>
       <c r="E168" s="1" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.2">
@@ -4803,7 +4803,7 @@
         <v>23</v>
       </c>
       <c r="E169" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.2">
@@ -4820,7 +4820,7 @@
         <v>25</v>
       </c>
       <c r="E170" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.2">
@@ -4837,7 +4837,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.2">
@@ -4854,7 +4854,7 @@
         <v>29</v>
       </c>
       <c r="E172" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.2">
@@ -4871,7 +4871,7 @@
         <v>31</v>
       </c>
       <c r="E173" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.2">
@@ -4888,7 +4888,7 @@
         <v>33</v>
       </c>
       <c r="E174" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.2">
@@ -4905,7 +4905,7 @@
         <v>35</v>
       </c>
       <c r="E175" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.2">
@@ -4922,7 +4922,7 @@
         <v>37</v>
       </c>
       <c r="E176" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.2">
@@ -4939,7 +4939,7 @@
         <v>232</v>
       </c>
       <c r="E177" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.2">
@@ -4956,7 +4956,7 @@
         <v>43</v>
       </c>
       <c r="E178" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.2">
@@ -4973,7 +4973,7 @@
         <v>45</v>
       </c>
       <c r="E179" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.2">
@@ -4990,7 +4990,7 @@
         <v>47</v>
       </c>
       <c r="E180" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.2">
@@ -5007,7 +5007,7 @@
         <v>49</v>
       </c>
       <c r="E181" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.2">
@@ -5024,7 +5024,7 @@
         <v>51</v>
       </c>
       <c r="E182" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.2">
@@ -5041,7 +5041,7 @@
         <v>53</v>
       </c>
       <c r="E183" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.2">
@@ -5058,7 +5058,7 @@
         <v>55</v>
       </c>
       <c r="E184" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.2">
@@ -5075,7 +5075,7 @@
         <v>57</v>
       </c>
       <c r="E185" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.2">
@@ -5092,7 +5092,7 @@
         <v>59</v>
       </c>
       <c r="E186" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.2">
@@ -5109,7 +5109,7 @@
         <v>61</v>
       </c>
       <c r="E187" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.2">
@@ -5126,7 +5126,7 @@
         <v>63</v>
       </c>
       <c r="E188" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.2">
@@ -5143,7 +5143,7 @@
         <v>65</v>
       </c>
       <c r="E189" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.2">
@@ -5160,7 +5160,7 @@
         <v>67</v>
       </c>
       <c r="E190" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.2">
@@ -5177,7 +5177,7 @@
         <v>69</v>
       </c>
       <c r="E191" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.2">
@@ -5194,7 +5194,7 @@
         <v>71</v>
       </c>
       <c r="E192" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.2">
@@ -5211,7 +5211,7 @@
         <v>73</v>
       </c>
       <c r="E193" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.2">
@@ -5228,7 +5228,7 @@
         <v>75</v>
       </c>
       <c r="E194" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.2">
@@ -5245,7 +5245,7 @@
         <v>77</v>
       </c>
       <c r="E195" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.2">
@@ -5262,7 +5262,7 @@
         <v>79</v>
       </c>
       <c r="E196" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.2">
@@ -5279,7 +5279,7 @@
         <v>81</v>
       </c>
       <c r="E197" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.2">
@@ -5296,7 +5296,7 @@
         <v>83</v>
       </c>
       <c r="E198" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.2">
@@ -5313,7 +5313,7 @@
         <v>85</v>
       </c>
       <c r="E199" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.2">
@@ -5330,7 +5330,7 @@
         <v>87</v>
       </c>
       <c r="E200" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.2">
@@ -5347,7 +5347,7 @@
         <v>89</v>
       </c>
       <c r="E201" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.2">
@@ -5364,7 +5364,7 @@
         <v>91</v>
       </c>
       <c r="E202" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.2">
@@ -5381,7 +5381,7 @@
         <v>93</v>
       </c>
       <c r="E203" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.2">
@@ -5398,7 +5398,7 @@
         <v>95</v>
       </c>
       <c r="E204" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.2">
@@ -5415,7 +5415,7 @@
         <v>97</v>
       </c>
       <c r="E205" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.2">
@@ -5432,7 +5432,7 @@
         <v>99</v>
       </c>
       <c r="E206" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.2">
@@ -5449,7 +5449,7 @@
         <v>101</v>
       </c>
       <c r="E207" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.2">
@@ -5466,7 +5466,7 @@
         <v>103</v>
       </c>
       <c r="E208" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.2">
@@ -5483,7 +5483,7 @@
         <v>105</v>
       </c>
       <c r="E209" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.2">
@@ -5500,7 +5500,7 @@
         <v>107</v>
       </c>
       <c r="E210" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.2">
@@ -5517,7 +5517,7 @@
         <v>109</v>
       </c>
       <c r="E211" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.2">
@@ -5534,7 +5534,7 @@
         <v>111</v>
       </c>
       <c r="E212" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.2">
@@ -5551,7 +5551,7 @@
         <v>113</v>
       </c>
       <c r="E213" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.2">
@@ -5568,7 +5568,7 @@
         <v>115</v>
       </c>
       <c r="E214" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.2">
@@ -5585,7 +5585,7 @@
         <v>117</v>
       </c>
       <c r="E215" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.2">
@@ -5602,7 +5602,7 @@
         <v>119</v>
       </c>
       <c r="E216" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.2">
@@ -5619,7 +5619,7 @@
         <v>121</v>
       </c>
       <c r="E217" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.2">
@@ -5636,7 +5636,7 @@
         <v>123</v>
       </c>
       <c r="E218" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.2">
@@ -5653,7 +5653,7 @@
         <v>125</v>
       </c>
       <c r="E219" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.2">
@@ -5670,7 +5670,7 @@
         <v>125</v>
       </c>
       <c r="E220" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.2">
@@ -5687,7 +5687,7 @@
         <v>128</v>
       </c>
       <c r="E221" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.2">
@@ -5704,7 +5704,7 @@
         <v>130</v>
       </c>
       <c r="E222" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.2">
@@ -5721,7 +5721,7 @@
         <v>132</v>
       </c>
       <c r="E223" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.2">
@@ -5738,7 +5738,7 @@
         <v>134</v>
       </c>
       <c r="E224" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.2">
@@ -5755,7 +5755,7 @@
         <v>136</v>
       </c>
       <c r="E225" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.2">
@@ -5766,7 +5766,7 @@
         <v>0</v>
       </c>
       <c r="E226" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.2">
@@ -5823,7 +5823,7 @@
         <v>233</v>
       </c>
       <c r="E230" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.2">
@@ -5840,7 +5840,7 @@
         <v>234</v>
       </c>
       <c r="E231" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="232" spans="1:5" x14ac:dyDescent="0.2">
@@ -5888,7 +5888,7 @@
         <v>461</v>
       </c>
       <c r="E234" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.2">
@@ -5975,7 +5975,7 @@
         <v>244</v>
       </c>
       <c r="E240" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.2">
@@ -6167,7 +6167,7 @@
         <v>251</v>
       </c>
       <c r="E252" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.2">
@@ -6328,7 +6328,7 @@
         <v>257</v>
       </c>
       <c r="E262" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="263" spans="1:5" x14ac:dyDescent="0.2">
@@ -6345,7 +6345,7 @@
         <v>258</v>
       </c>
       <c r="E263" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="264" spans="1:5" x14ac:dyDescent="0.2">
@@ -6413,7 +6413,7 @@
         <v>262</v>
       </c>
       <c r="E267" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="268" spans="1:5" x14ac:dyDescent="0.2">
@@ -6430,7 +6430,7 @@
         <v>263</v>
       </c>
       <c r="E268" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="269" spans="1:5" x14ac:dyDescent="0.2">
@@ -6617,7 +6617,7 @@
         <v>270</v>
       </c>
       <c r="E282" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
   </sheetData>

</xml_diff>